<commit_message>
Updated BOM /Round LED 1, Square_Board 1,Touch board 1
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Altium_Generated/LED_Square_1.xlsx
+++ b/Deliverables/BOM/Altium_Generated/LED_Square_1.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\IbrahimHyder-ReverseEngineering\Deliverables\BOM\Altium_Generated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\IbrahimHyder-ReverseEngineering\Deliverables\BOM\Altium_Generated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36635F7E-187F-4E90-A75F-055793BFBDA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="300" windowWidth="10335" windowHeight="10620" xr2:uid="{CD259ABF-650E-4745-BD8A-5FABD9A9E960}"/>
+    <workbookView xWindow="2685" yWindow="300" windowWidth="10335" windowHeight="10620"/>
   </bookViews>
   <sheets>
     <sheet name="LED_Square_1" sheetId="1" r:id="rId1"/>
@@ -114,7 +113,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -490,7 +489,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCF89A03-ECC8-43B3-8682-2187C5634AD2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>